<commit_message>
Actualizacao dos desistentes e graficos  ambientais
</commit_message>
<xml_diff>
--- a/EMPREENDEDORAS_PAM_VERDE_C3_2026.xlsx
+++ b/EMPREENDEDORAS_PAM_VERDE_C3_2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30306"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30317"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://muvamozorg.sharepoint.com/sites/mis.drive/Documentos Partilhados/PROJECTOS/Sistema de Monitoria/Pam_Verde/2026/Baseline_Endline/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="204" documentId="11_0DFBC18E49307CB38E73D6987E34D4946C7A7096" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{F8496164-C0E2-4DFD-956E-A06726BA187B}"/>
+  <xr:revisionPtr revIDLastSave="214" documentId="11_0DFBC18E49307CB38E73D6987E34D4946C7A7096" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{51DD1827-C1A9-4E58-9E3D-30F2E4BA369D}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -36,7 +36,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4294" uniqueCount="1185">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="4297" uniqueCount="1186">
   <si>
     <t>Confirma que compreendeu a informação acima e aceita participar nesta entrevista?</t>
   </si>
@@ -3777,6 +3777,9 @@
   </si>
   <si>
     <t>Por motivo de Doenca (Passa para o proximo ciclo)</t>
+  </si>
+  <si>
+    <t>Passa para proximo ciclo</t>
   </si>
   <si>
     <t>PAM_2026_52</t>
@@ -3889,7 +3892,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="3">
+  <fills count="4">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -3899,6 +3902,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor rgb="FFFF0000"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFFF00"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -3915,7 +3924,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="9">
+  <cellXfs count="10">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
     <xf numFmtId="1" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -3925,6 +3934,7 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="1" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="0" fillId="3" borderId="0" xfId="0" applyFill="1"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -4369,7 +4379,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:CJ51"/>
+  <dimension ref="A1:CL51"/>
   <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
     <col min="1" max="3" width="16" hidden="1" customWidth="1"/>
@@ -8617,7 +8627,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="17" spans="1:88">
+    <row r="17" spans="1:90">
       <c r="A17" t="s">
         <v>88</v>
       </c>
@@ -8880,7 +8890,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="18" spans="1:88">
+    <row r="18" spans="1:90">
       <c r="A18" t="s">
         <v>88</v>
       </c>
@@ -9143,7 +9153,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="19" spans="1:88">
+    <row r="19" spans="1:90">
       <c r="A19" t="s">
         <v>88</v>
       </c>
@@ -9406,7 +9416,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="20" spans="1:88">
+    <row r="20" spans="1:90">
       <c r="A20" t="s">
         <v>88</v>
       </c>
@@ -9672,7 +9682,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="21" spans="1:88">
+    <row r="21" spans="1:90">
       <c r="A21" t="s">
         <v>88</v>
       </c>
@@ -9935,7 +9945,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="22" spans="1:88">
+    <row r="22" spans="1:90">
       <c r="A22" t="s">
         <v>88</v>
       </c>
@@ -10198,8 +10208,9 @@
       <c r="CJ22" t="s">
         <v>466</v>
       </c>
+      <c r="CL22" s="9"/>
     </row>
-    <row r="23" spans="1:88">
+    <row r="23" spans="1:90">
       <c r="A23" t="s">
         <v>88</v>
       </c>
@@ -10462,7 +10473,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="24" spans="1:88">
+    <row r="24" spans="1:90">
       <c r="A24" t="s">
         <v>88</v>
       </c>
@@ -10725,7 +10736,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="25" spans="1:88">
+    <row r="25" spans="1:90">
       <c r="A25" t="s">
         <v>88</v>
       </c>
@@ -10988,7 +10999,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="26" spans="1:88">
+    <row r="26" spans="1:90">
       <c r="A26" t="s">
         <v>88</v>
       </c>
@@ -11251,7 +11262,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="27" spans="1:88">
+    <row r="27" spans="1:90">
       <c r="A27" t="s">
         <v>88</v>
       </c>
@@ -11517,7 +11528,7 @@
         <v>144</v>
       </c>
     </row>
-    <row r="28" spans="1:88">
+    <row r="28" spans="1:90">
       <c r="A28" t="s">
         <v>88</v>
       </c>
@@ -11781,7 +11792,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="29" spans="1:88">
+    <row r="29" spans="1:90">
       <c r="A29" t="s">
         <v>88</v>
       </c>
@@ -12044,7 +12055,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="30" spans="1:88">
+    <row r="30" spans="1:90">
       <c r="A30" t="s">
         <v>88</v>
       </c>
@@ -12307,7 +12318,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="31" spans="1:88">
+    <row r="31" spans="1:90">
       <c r="A31" t="s">
         <v>88</v>
       </c>
@@ -12571,7 +12582,7 @@
         <v>466</v>
       </c>
     </row>
-    <row r="32" spans="1:88">
+    <row r="32" spans="1:90">
       <c r="A32" t="s">
         <v>88</v>
       </c>
@@ -17048,7 +17059,7 @@
         <v>177</v>
       </c>
     </row>
-    <row r="49" spans="1:88">
+    <row r="49" spans="1:90">
       <c r="A49" t="s">
         <v>88</v>
       </c>
@@ -17313,8 +17324,11 @@
       <c r="CJ49" t="s">
         <v>144</v>
       </c>
+      <c r="CL49" s="9" t="s">
+        <v>1161</v>
+      </c>
     </row>
-    <row r="50" spans="1:88">
+    <row r="50" spans="1:90">
       <c r="A50" t="s">
         <v>88</v>
       </c>
@@ -17331,10 +17345,10 @@
         <v>91</v>
       </c>
       <c r="F50" s="3" t="s">
-        <v>1161</v>
+        <v>1162</v>
       </c>
       <c r="G50" s="3" t="s">
-        <v>1162</v>
+        <v>1163</v>
       </c>
       <c r="H50" s="3" t="s">
         <v>94</v>
@@ -17355,7 +17369,7 @@
         <v>106</v>
       </c>
       <c r="N50" s="3" t="s">
-        <v>1163</v>
+        <v>1164</v>
       </c>
       <c r="O50" s="3" t="s">
         <v>100</v>
@@ -17397,7 +17411,7 @@
         <v>108</v>
       </c>
       <c r="AB50" s="3" t="s">
-        <v>1164</v>
+        <v>1165</v>
       </c>
       <c r="AC50" s="3" t="s">
         <v>154</v>
@@ -17454,22 +17468,22 @@
         <v>106</v>
       </c>
       <c r="AU50" s="3" t="s">
-        <v>1165</v>
+        <v>1166</v>
       </c>
       <c r="AV50" s="3" t="s">
         <v>120</v>
       </c>
       <c r="AW50" s="3" t="s">
-        <v>1166</v>
+        <v>1167</v>
       </c>
       <c r="AX50" s="3" t="s">
-        <v>1167</v>
+        <v>1168</v>
       </c>
       <c r="AY50" s="3" t="s">
-        <v>1168</v>
+        <v>1169</v>
       </c>
       <c r="AZ50" s="3" t="s">
-        <v>1169</v>
+        <v>1170</v>
       </c>
       <c r="BA50" s="3" t="s">
         <v>114</v>
@@ -17490,46 +17504,46 @@
         <v>125</v>
       </c>
       <c r="BG50" s="3" t="s">
-        <v>1170</v>
+        <v>1171</v>
       </c>
       <c r="BH50" s="3" t="s">
-        <v>1171</v>
+        <v>1172</v>
       </c>
       <c r="BI50" s="3" t="s">
         <v>167</v>
       </c>
       <c r="BJ50" s="3" t="s">
-        <v>1172</v>
+        <v>1173</v>
       </c>
       <c r="BK50" s="3" t="s">
         <v>167</v>
       </c>
       <c r="BL50" s="3" t="s">
-        <v>1173</v>
+        <v>1174</v>
       </c>
       <c r="BM50" s="3" t="s">
         <v>128</v>
       </c>
       <c r="BN50" s="3" t="s">
-        <v>1174</v>
+        <v>1175</v>
       </c>
       <c r="BO50" s="3" t="s">
         <v>128</v>
       </c>
       <c r="BP50" s="3" t="s">
-        <v>1175</v>
+        <v>1176</v>
       </c>
       <c r="BQ50" s="3" t="s">
         <v>128</v>
       </c>
       <c r="BR50" s="3" t="s">
-        <v>1176</v>
+        <v>1177</v>
       </c>
       <c r="BS50" s="3" t="s">
         <v>130</v>
       </c>
       <c r="BT50" s="3" t="s">
-        <v>1177</v>
+        <v>1178</v>
       </c>
       <c r="BU50" s="3" t="s">
         <v>128</v>
@@ -17544,10 +17558,10 @@
         <v>138</v>
       </c>
       <c r="BY50" s="3" t="s">
-        <v>1178</v>
+        <v>1179</v>
       </c>
       <c r="BZ50" s="3" t="s">
-        <v>1179</v>
+        <v>1180</v>
       </c>
       <c r="CA50" s="3" t="s">
         <v>102</v>
@@ -17568,28 +17582,31 @@
         <v>227</v>
       </c>
       <c r="CG50" s="3" t="s">
-        <v>1180</v>
+        <v>1181</v>
       </c>
       <c r="CH50" s="3" t="s">
         <v>142</v>
       </c>
       <c r="CI50" s="3" t="s">
-        <v>1181</v>
+        <v>1182</v>
       </c>
       <c r="CJ50" t="s">
         <v>144</v>
       </c>
+      <c r="CL50" s="9" t="s">
+        <v>1161</v>
+      </c>
     </row>
-    <row r="51" spans="1:88">
+    <row r="51" spans="1:90">
       <c r="B51" s="1"/>
       <c r="E51" s="3" t="s">
         <v>91</v>
       </c>
       <c r="F51" s="3" t="s">
-        <v>1182</v>
+        <v>1183</v>
       </c>
       <c r="G51" s="3" t="s">
-        <v>1183</v>
+        <v>1184</v>
       </c>
       <c r="H51" s="3" t="s">
         <v>94</v>
@@ -17827,10 +17844,13 @@
       </c>
       <c r="CH51" s="3"/>
       <c r="CI51" s="3" t="s">
-        <v>1184</v>
+        <v>1185</v>
       </c>
       <c r="CJ51" t="s">
         <v>144</v>
+      </c>
+      <c r="CL51" s="9" t="s">
+        <v>1161</v>
       </c>
     </row>
   </sheetData>
@@ -17842,15 +17862,6 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
-</file>
-
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
   <documentManagement>
     <TaxCatchAll xmlns="54c5ab46-7543-4aba-b0fa-79d6a199bef5" xsi:nil="true"/>
@@ -17861,7 +17872,7 @@
 </p:properties>
 </file>
 
-<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Documento" ma:contentTypeID="0x010100DC8BB5B596CFDD4794B3344F0E8F53A4" ma:contentTypeVersion="15" ma:contentTypeDescription="Criar um novo documento." ma:contentTypeScope="" ma:versionID="9a7078cd21229583650f2264465a1c40">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:ns2="20d57abc-823c-4051-a81a-1a0a01a8f39e" xmlns:ns3="54c5ab46-7543-4aba-b0fa-79d6a199bef5" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="4e45437c47114f519c494620e3e4bb67" ns2:_="" ns3:_="">
     <xsd:import namespace="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
@@ -18096,14 +18107,23 @@
 </ct:contentTypeSchema>
 </file>
 
+<file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
+</file>
+
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E5422FBB-6025-4E11-8C1C-C4A520C0A5F3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6C6D4B0-20F6-407F-B938-614BBBC09F61}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6C6D4B0-20F6-407F-B938-614BBBC09F61}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA033CCE-4348-4253-93A3-12EE2F84ACE6}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{CA033CCE-4348-4253-93A3-12EE2F84ACE6}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E5422FBB-6025-4E11-8C1C-C4A520C0A5F3}"/>
 </file>
</xml_diff>

<commit_message>
Actualizacao das paginas da Beira
</commit_message>
<xml_diff>
--- a/EMPREENDEDORAS_PAM_VERDE_C3_2026.xlsx
+++ b/EMPREENDEDORAS_PAM_VERDE_C3_2026.xlsx
@@ -1,14 +1,14 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30317"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="30327"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://muvamozorg.sharepoint.com/sites/mis.drive/Documentos Partilhados/PROJECTOS/Sistema de Monitoria/Pam_Verde/2026/Baseline_Endline/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="214" documentId="11_0DFBC18E49307CB38E73D6987E34D4946C7A7096" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{51DD1827-C1A9-4E58-9E3D-30F2E4BA369D}"/>
+  <xr:revisionPtr revIDLastSave="215" documentId="11_0DFBC18E49307CB38E73D6987E34D4946C7A7096" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{662CF095-CF90-40A3-9454-44CB2AA9DD0A}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -4387,16 +4387,16 @@
     <col min="5" max="5" width="19" bestFit="1" customWidth="1"/>
     <col min="6" max="6" width="22.85546875" customWidth="1"/>
     <col min="7" max="7" width="38" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="9" hidden="1" customWidth="1"/>
-    <col min="9" max="9" width="16" hidden="1" customWidth="1"/>
-    <col min="10" max="10" width="13" hidden="1" customWidth="1"/>
-    <col min="11" max="16" width="16" hidden="1" customWidth="1"/>
-    <col min="17" max="17" width="23.7109375" hidden="1" customWidth="1"/>
-    <col min="18" max="24" width="16" hidden="1" customWidth="1"/>
-    <col min="25" max="25" width="8" hidden="1" customWidth="1"/>
-    <col min="26" max="72" width="16" hidden="1" customWidth="1"/>
-    <col min="73" max="73" width="14" hidden="1" customWidth="1"/>
-    <col min="74" max="85" width="16" hidden="1" customWidth="1"/>
+    <col min="8" max="8" width="9" customWidth="1"/>
+    <col min="9" max="9" width="16" customWidth="1"/>
+    <col min="10" max="10" width="13" customWidth="1"/>
+    <col min="11" max="16" width="16" customWidth="1"/>
+    <col min="17" max="17" width="23.7109375" customWidth="1"/>
+    <col min="18" max="24" width="16" customWidth="1"/>
+    <col min="25" max="25" width="8" customWidth="1"/>
+    <col min="26" max="72" width="16" customWidth="1"/>
+    <col min="73" max="73" width="14" customWidth="1"/>
+    <col min="74" max="85" width="16" customWidth="1"/>
     <col min="86" max="86" width="29.85546875" customWidth="1"/>
     <col min="87" max="87" width="65.85546875" customWidth="1"/>
     <col min="88" max="88" width="11" bestFit="1" customWidth="1"/>
@@ -17862,14 +17862,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="54c5ab46-7543-4aba-b0fa-79d6a199bef5" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="20d57abc-823c-4051-a81a-1a0a01a8f39e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -18108,16 +18106,18 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="54c5ab46-7543-4aba-b0fa-79d6a199bef5" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="20d57abc-823c-4051-a81a-1a0a01a8f39e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6C6D4B0-20F6-407F-B938-614BBBC09F61}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E5422FBB-6025-4E11-8C1C-C4A520C0A5F3}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -18125,5 +18125,5 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E5422FBB-6025-4E11-8C1C-C4A520C0A5F3}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6C6D4B0-20F6-407F-B938-614BBBC09F61}"/>
 </file>
</xml_diff>

<commit_message>
Actualizacao dos exercicios do endline
</commit_message>
<xml_diff>
--- a/EMPREENDEDORAS_PAM_VERDE_C3_2026.xlsx
+++ b/EMPREENDEDORAS_PAM_VERDE_C3_2026.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://muvamozorg.sharepoint.com/sites/mis.drive/Documentos Partilhados/PROJECTOS/Sistema de Monitoria/Pam_Verde/2026/Baseline_Endline/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="223" documentId="11_0DFBC18E49307CB38E73D6987E34D4946C7A7096" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{BEA4346B-BC59-4905-9F83-CF1A73DB274E}"/>
+  <xr:revisionPtr revIDLastSave="225" documentId="11_0DFBC18E49307CB38E73D6987E34D4946C7A7096" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{D722354E-BFC5-4D44-9CC1-B7C001EF276D}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="14295" yWindow="0" windowWidth="14610" windowHeight="15585" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Empreendedoras_Nampula_C3_2026" sheetId="1" r:id="rId1"/>
@@ -17863,14 +17863,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement>
-    <TaxCatchAll xmlns="54c5ab46-7543-4aba-b0fa-79d6a199bef5" xsi:nil="true"/>
-    <lcf76f155ced4ddcb4097134ff3c332f xmlns="20d57abc-823c-4051-a81a-1a0a01a8f39e">
-      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    </lcf76f155ced4ddcb4097134ff3c332f>
-  </documentManagement>
-</p:properties>
+<?mso-contentType ?>
+<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
+  <Display>DocumentLibraryForm</Display>
+  <Edit>DocumentLibraryForm</Edit>
+  <New>DocumentLibraryForm</New>
+</FormTemplates>
 </file>
 
 <file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
@@ -18109,21 +18107,20 @@
 </file>
 
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
-<?mso-contentType ?>
-<FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
-  <Display>DocumentLibraryForm</Display>
-  <Edit>DocumentLibraryForm</Edit>
-  <New>DocumentLibraryForm</New>
-</FormTemplates>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement>
+    <TaxCatchAll xmlns="54c5ab46-7543-4aba-b0fa-79d6a199bef5" xsi:nil="true"/>
+    <lcf76f155ced4ddcb4097134ff3c332f xmlns="20d57abc-823c-4051-a81a-1a0a01a8f39e">
+      <Terms xmlns="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    </lcf76f155ced4ddcb4097134ff3c332f>
+  </documentManagement>
+</p:properties>
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6C6D4B0-20F6-407F-B938-614BBBC09F61}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E5422FBB-6025-4E11-8C1C-C4A520C0A5F3}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="54c5ab46-7543-4aba-b0fa-79d6a199bef5"/>
-    <ds:schemaRef ds:uri="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
@@ -18148,9 +18145,12 @@
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{E5422FBB-6025-4E11-8C1C-C4A520C0A5F3}">
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{F6C6D4B0-20F6-407F-B938-614BBBC09F61}">
   <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="54c5ab46-7543-4aba-b0fa-79d6a199bef5"/>
+    <ds:schemaRef ds:uri="20d57abc-823c-4051-a81a-1a0a01a8f39e"/>
   </ds:schemaRefs>
 </ds:datastoreItem>
 </file>
</xml_diff>